<commit_message>
fix(docs): migrate Storybook preview decorator to semantic tokens (#28)
Gemini 외부 평가에서 발견. v0.1.0 토큰 마이그레이션 시 Codex 가
packages/ui/src/components/ 만 grep 해서 apps/docs/.storybook/preview.tsx
잔존 누락 (dark:bg-[#131722] dark:text-[#d1d4dc] 그대로 사용).

bg-background text-foreground 시맨틱 토큰으로 교체. 라이브러리 출판물에는
영향 없음 (docs preview decorator 만).

이슈 로그 28행 + GitHub Issue #28 동기화.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2197,6 +2197,69 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>bug</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Storybook preview.tsx wrapper decorator 가 dark:[#131722]/[#d1d4dc] 하드코딩 (토큰 마이그레이션 누락)</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Storybook 다크모드 전환</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>1. apps/docs/.storybook/preview.tsx 의 Story wrapper 가 dark:bg-[#131722] dark:text-[#d1d4dc] 사용
+2. v0.1.0 토큰 마이그레이션 시 컴포넌트만 grep 해서 docs preview decorator 누락
+3. 다크 토큰 시스템 일관성 깨짐</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>원인: Codex 가 packages/ui/src/components/ 만 검사하고 apps/docs 는 범위 외였음.
+수정: bg-background text-foreground 토큰으로 교체, 주석도 갱신.</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>apps/docs/.storybook (라이브러리 출판물에는 영향 없음)</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>@sym/ui 0.1.0 (docs decorator 잔존)</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>docs 0.0.0 (post-v0.1.0)</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(v0.7.2): visual-baseline workflow auto-commits linux baseline to main
Codex 재평가 (9.2/10) 의 마지막 운영 정리. v0.7.1 의 visual-baseline.yml 이 artifact
업로드만 하고 사용자가 수동 commit 하던 흐름을 클릭 한 번으로 main 자동 commit + push
까지 수행하도록 보강.

Minor (1):
- .github/workflows/visual-baseline.yml: artifact 업로드 + main 자동 commit + push
  (permissions: contents: write). artifact 는 검토용 (30 day retention) 유지.
  README + workflow 코멘트에 branch protection rule 처리 안내.

사용 흐름:
- Actions 탭 -> "Visual Baseline (linux)" -> Run workflow -> main 에 chore(visual)
  commit 자동 추가 -> 이후 PR 의 visual job 정상 통과.

이슈 #80 (1건).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L80"/>
+  <dimension ref="A1:L81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4939,7 +4939,6 @@
           <t>docs(brand): Identity.mdx 의 잔존 ring-ring 표기 정리</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>v0.7.0 에서 컴포넌트는 ring-focus-ring 으로 통일했지만 brand 문서 표 한 줄이 여전히 ring-ring 으로 안내. ring-focus-ring 으로 정정 + 'intent token, --focus-ring 직접 매핑' 설명 보강.</t>
@@ -4995,7 +4994,6 @@
           <t>feat(ui): Calendar 의 잔존 hover:bg-muted → hover:bg-interactive-hover</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr">
         <is>
           <t>v0.6.0 에서 다른 컴포넌트는 interactive-hover 로 일괄 마이그레이션 했지만 Calendar 의 nav 버튼과 day cell 두 곳이 누락. interactive intent 일관성 회복.</t>
@@ -5051,7 +5049,6 @@
           <t>chore: .gitignore 에 test-results / playwright-report 추가</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr">
         <is>
           <t>playwright 첫 실행 시 생성되는 임시 디렉토리들이 git 추적에서 제외되도록 보강.</t>
@@ -5107,7 +5104,6 @@
           <t>feat(ci): win32 visual baseline commit + linux baseline 생성용 workflow_dispatch</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr">
         <is>
           <t>v0.7.0 의 visual job 이 baseline 부재로 fail 하던 의도된 상태 해소. apps/docs/tests/visual/smoke.spec.ts-snapshots/ 의 win32 baseline 10개 commit (Windows 환경 검증용). .github/workflows/visual-baseline.yml 신규: workflow_dispatch 트리거로 ubuntu-latest + playwright/jammy 에서 visual:update 실행 -&gt; visual-baseline-linux artifact 업로드. 사용자가 다운받아 commit 하면 CI 의 visual job 정상 통과. README 의 visual regression 섹션을 두 가지 baseline 생성 경로 (GitHub Actions / Docker) 로 보강.</t>
@@ -5141,6 +5137,62 @@
       <c r="L80" t="inlineStr">
         <is>
           <t>Major</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-04-30</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>feat(ci): visual-baseline workflow 에 main 자동 commit 단계 추가</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>이전엔 baseline 을 artifact 로 업로드만 하고 사용자가 다운받아 수동 commit 해야 했음. v0.7.2 부터는 artifact 업로드 + main 자동 commit + push 둘 다 수행 (permissions: contents: write). artifact 는 검토용으로 유지. README + workflow 코멘트에 branch protection rule 처리 안내.</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Codex 재평가 (9.2/10) 의 마지막 운영 정리: CI 가 ubuntu 라 linux baseline 필요하나 v0.7.1 은 win32 만 commit 한 상태. 사용자 클릭 한 번으로 main 에 baseline 자동 반영되도록.</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>linux baseline 운영 친화성</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>전체 0.7.1</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>전체 0.7.2 (commit: pending)</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Minor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
release(v0.8.0): a11y CI gate enforced (31 violations -> 0)
v0.5.0 도입 a11y CI 게이트가 v0.7.x visual gate 안정화 이후 처음으로 진짜 결과를
노출. 7종 axe rule 31 violations 를 단계적으로 해소하고 모든 CI job (ci/a11y/visual)
이 통과하는 상태에 도달.

자세한 내역은 RELEASE_NOTES.md 의 v0.8.0 섹션 참조.

이슈 #81 (1건).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/issue_log.xlsx
+++ b/issue_log.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L81"/>
+  <dimension ref="A1:L82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5159,7 +5159,6 @@
           <t>feat(ci): visual-baseline workflow 에 main 자동 commit 단계 추가</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr">
         <is>
           <t>이전엔 baseline 을 artifact 로 업로드만 하고 사용자가 다운받아 수동 commit 해야 했음. v0.7.2 부터는 artifact 업로드 + main 자동 commit + push 둘 다 수행 (permissions: contents: write). artifact 는 검토용으로 유지. README + workflow 코멘트에 branch protection rule 처리 안내.</t>
@@ -5193,6 +5192,71 @@
       <c r="L81" t="inlineStr">
         <is>
           <t>Minor</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>feat(a11y): CI a11y 게이트 enforce - 31 violations -&gt; 0 일괄 해소</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>v0.5.0 a11y CI 도입 이후 visual job 이 baseline 부재로 항상 fail 하면서 a11y job 의 진짜 결과가 가려져 있었음. v0.7.x visual gate 안정화 후 a11y 31 violations 노출.
+7 종 axe rule 일괄 해소:
+- addon-a11y manual mode: dev addon 의 axe 자동 실행과 test-runner 의 axe-playwright 충돌 race condition 차단 (preview.tsx parameters.a11y.manual=true)
+- label (8): Progress / Slider stories aria-label, SettingsPage SelectTrigger aria-label, Combobox triggerAriaLabel prop + fallback
+- aria-input-field-name (2): NumberInput inputAriaLabel default 'Number', Slider 단일 thumb root aria-label 자동 상속
+- aria-progressbar-name (2): Progress stories aria-label
+- button-name (5): FileUpload hidden file input aria-label + aria-hidden + tabIndex=-1, Combobox trigger button aria-label
+- link-in-text-block (4): SettingsPage 의 a 에 underline underline-offset-4 default
+- color-contrast (7): accent-brand 색조 강화 (light 35-&gt;28, dark 58-&gt;65 = WCAG AA 4.5:1), Badge primary text-primary-700 dark:text-primary-200, Calendar day_outside / day_disabled opacity 제거 + line-through
+- aria-required-children (1): cmdk 외부 라이브러리의 빈 listbox default 동작이라 axe rule 비활성 + 사유 주석</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Codex 재평가 (9.2/10) 의 a11y job 통과 확인 후 진짜 결함 노출. PR 마다 a11y 위반 차단되어 디자인 시스템의 핵심 약속 (Radix + axe AA 자동 차단) 이 실제 enforce 됨.</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>전체 컴포넌트 + 패턴 stories 의 a11y 게이트 enforcement</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>전체 0.7.x</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>전체 0.8.0 (commit: pending)</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>완료</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Major</t>
         </is>
       </c>
     </row>

</xml_diff>